<commit_message>
dos pines mal, ya esta la configuracion de pines en el controlador
</commit_message>
<xml_diff>
--- a/hardware/Circuito Final/Circuito externo/Pines controlador.xlsx
+++ b/hardware/Circuito Final/Circuito externo/Pines controlador.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="110">
   <si>
     <t>PC10</t>
   </si>
@@ -500,6 +500,21 @@
   </si>
   <si>
     <t>llave de emergencia</t>
+  </si>
+  <si>
+    <t>CLK</t>
+  </si>
+  <si>
+    <t>LATCH</t>
+  </si>
+  <si>
+    <t>S0</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>S2</t>
   </si>
 </sst>
 </file>
@@ -737,7 +752,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -791,12 +806,6 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -814,6 +823,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1047,40 +1065,40 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="27">
+      <c r="B2" s="25">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="E2" s="24" t="s">
-        <v>76</v>
+      <c r="D2" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>106</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="26">
+      <c r="G2" s="24">
         <v>1</v>
       </c>
-      <c r="I2" s="27">
+      <c r="I2" s="25">
         <v>2</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="L2" s="24" t="s">
-        <v>73</v>
+      <c r="K2" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="L2" s="30" t="s">
+        <v>108</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="26">
+      <c r="N2" s="24">
         <v>1</v>
       </c>
       <c r="P2" s="4" t="s">
@@ -1094,34 +1112,36 @@
       </c>
     </row>
     <row r="3" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="27">
+      <c r="B3" s="25">
         <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="16"/>
+      <c r="D3" s="16" t="s">
+        <v>5</v>
+      </c>
       <c r="E3" s="14"/>
       <c r="F3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="24">
         <v>3</v>
       </c>
-      <c r="I3" s="27">
+      <c r="I3" s="25">
         <v>4</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="K3" s="12"/>
-      <c r="L3" s="25" t="s">
-        <v>74</v>
+      <c r="L3" s="31" t="s">
+        <v>109</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="N3" s="26">
+      <c r="N3" s="24">
         <v>3</v>
       </c>
       <c r="P3" s="5" t="s">
@@ -1135,7 +1155,7 @@
       </c>
     </row>
     <row r="4" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="27">
+      <c r="B4" s="25">
         <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1146,10 +1166,10 @@
       <c r="F4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="24">
         <v>5</v>
       </c>
-      <c r="I4" s="27">
+      <c r="I4" s="25">
         <v>6</v>
       </c>
       <c r="J4" s="2" t="s">
@@ -1162,7 +1182,7 @@
       <c r="M4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N4" s="30">
+      <c r="N4" s="28">
         <v>5</v>
       </c>
       <c r="P4" s="6" t="s">
@@ -1176,7 +1196,7 @@
       </c>
     </row>
     <row r="5" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="27">
+      <c r="B5" s="25">
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1187,10 +1207,10 @@
       <c r="F5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="24">
         <v>7</v>
       </c>
-      <c r="I5" s="27">
+      <c r="I5" s="25">
         <v>8</v>
       </c>
       <c r="J5" s="2" t="s">
@@ -1201,7 +1221,7 @@
       <c r="M5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N5" s="26">
+      <c r="N5" s="24">
         <v>7</v>
       </c>
       <c r="P5" s="7" t="s">
@@ -1215,7 +1235,7 @@
       </c>
     </row>
     <row r="6" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="27">
+      <c r="B6" s="25">
         <v>10</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -1226,10 +1246,10 @@
       <c r="F6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="26">
+      <c r="G6" s="24">
         <v>9</v>
       </c>
-      <c r="I6" s="27">
+      <c r="I6" s="25">
         <v>10</v>
       </c>
       <c r="J6" s="2" t="s">
@@ -1240,7 +1260,7 @@
       <c r="M6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="26">
+      <c r="N6" s="24">
         <v>9</v>
       </c>
       <c r="P6" s="8" t="s">
@@ -1254,7 +1274,7 @@
       </c>
     </row>
     <row r="7" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="27">
+      <c r="B7" s="25">
         <v>12</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -1265,10 +1285,10 @@
       <c r="F7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="26">
+      <c r="G7" s="24">
         <v>11</v>
       </c>
-      <c r="I7" s="29">
+      <c r="I7" s="27">
         <v>12</v>
       </c>
       <c r="J7" s="2" t="s">
@@ -1277,13 +1297,13 @@
       <c r="K7" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="L7" s="25" t="s">
+      <c r="L7" s="23" t="s">
         <v>79</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="N7" s="26">
+      <c r="N7" s="24">
         <v>11</v>
       </c>
       <c r="P7" s="9" t="s">
@@ -1297,23 +1317,21 @@
       </c>
     </row>
     <row r="8" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="27">
+      <c r="B8" s="25">
         <v>14</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="28" t="s">
-        <v>5</v>
-      </c>
+      <c r="D8" s="26"/>
       <c r="E8" s="14"/>
       <c r="F8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="24">
         <v>13</v>
       </c>
-      <c r="I8" s="27">
+      <c r="I8" s="25">
         <v>14</v>
       </c>
       <c r="J8" s="2" t="s">
@@ -1322,13 +1340,13 @@
       <c r="K8" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="L8" s="25" t="s">
+      <c r="L8" s="23" t="s">
         <v>78</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N8" s="26">
+      <c r="N8" s="24">
         <v>13</v>
       </c>
       <c r="S8" s="21" t="s">
@@ -1339,7 +1357,7 @@
       </c>
     </row>
     <row r="9" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="27">
+      <c r="B9" s="25">
         <v>16</v>
       </c>
       <c r="C9" s="11" t="s">
@@ -1352,10 +1370,10 @@
       <c r="F9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="26">
+      <c r="G9" s="24">
         <v>15</v>
       </c>
-      <c r="I9" s="29">
+      <c r="I9" s="27">
         <v>16</v>
       </c>
       <c r="J9" s="2" t="s">
@@ -1368,7 +1386,7 @@
       <c r="M9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N9" s="26">
+      <c r="N9" s="24">
         <v>15</v>
       </c>
       <c r="S9" s="21" t="s">
@@ -1379,21 +1397,23 @@
       </c>
     </row>
     <row r="10" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="27">
+      <c r="B10" s="25">
         <v>18</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="16" t="s">
+        <v>37</v>
+      </c>
       <c r="E10" s="14"/>
       <c r="F10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="26">
+      <c r="G10" s="24">
         <v>17</v>
       </c>
-      <c r="I10" s="27">
+      <c r="I10" s="25">
         <v>18</v>
       </c>
       <c r="J10" s="2" t="s">
@@ -1404,7 +1424,7 @@
       <c r="M10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N10" s="26">
+      <c r="N10" s="24">
         <v>17</v>
       </c>
       <c r="S10" s="21" t="s">
@@ -1415,7 +1435,7 @@
       </c>
     </row>
     <row r="11" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="27">
+      <c r="B11" s="25">
         <v>20</v>
       </c>
       <c r="C11" s="11" t="s">
@@ -1426,10 +1446,10 @@
       <c r="F11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="26">
+      <c r="G11" s="24">
         <v>19</v>
       </c>
-      <c r="I11" s="27">
+      <c r="I11" s="25">
         <v>20</v>
       </c>
       <c r="J11" s="2" t="s">
@@ -1440,7 +1460,7 @@
       <c r="M11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="26">
+      <c r="N11" s="24">
         <v>19</v>
       </c>
       <c r="S11" s="21" t="s">
@@ -1451,7 +1471,7 @@
       </c>
     </row>
     <row r="12" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="27">
+      <c r="B12" s="25">
         <v>22</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -1462,10 +1482,10 @@
       <c r="F12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="26">
+      <c r="G12" s="24">
         <v>21</v>
       </c>
-      <c r="I12" s="27">
+      <c r="I12" s="25">
         <v>22</v>
       </c>
       <c r="J12" s="2" t="s">
@@ -1476,7 +1496,7 @@
       <c r="M12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="N12" s="26">
+      <c r="N12" s="24">
         <v>21</v>
       </c>
       <c r="T12" s="21" t="s">
@@ -1484,23 +1504,21 @@
       </c>
     </row>
     <row r="13" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="27">
+      <c r="B13" s="25">
         <v>24</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="28" t="s">
-        <v>37</v>
-      </c>
+      <c r="D13" s="26"/>
       <c r="E13" s="14"/>
       <c r="F13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G13" s="26">
+      <c r="G13" s="24">
         <v>23</v>
       </c>
-      <c r="I13" s="27">
+      <c r="I13" s="25">
         <v>24</v>
       </c>
       <c r="J13" s="2" t="s">
@@ -1511,7 +1529,7 @@
       <c r="M13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="N13" s="26">
+      <c r="N13" s="24">
         <v>23</v>
       </c>
       <c r="T13" s="21" t="s">
@@ -1519,7 +1537,7 @@
       </c>
     </row>
     <row r="14" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="27">
+      <c r="B14" s="25">
         <v>26</v>
       </c>
       <c r="C14" s="11" t="s">
@@ -1530,10 +1548,10 @@
       <c r="F14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="26">
+      <c r="G14" s="24">
         <v>25</v>
       </c>
-      <c r="I14" s="27">
+      <c r="I14" s="25">
         <v>26</v>
       </c>
       <c r="J14" s="2" t="s">
@@ -1544,7 +1562,7 @@
       <c r="M14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="N14" s="26">
+      <c r="N14" s="24">
         <v>25</v>
       </c>
       <c r="T14" s="21" t="s">
@@ -1552,7 +1570,7 @@
       </c>
     </row>
     <row r="15" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="27">
+      <c r="B15" s="25">
         <v>28</v>
       </c>
       <c r="C15" s="11" t="s">
@@ -1565,10 +1583,10 @@
       <c r="F15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G15" s="30">
+      <c r="G15" s="28">
         <v>27</v>
       </c>
-      <c r="I15" s="27">
+      <c r="I15" s="25">
         <v>28</v>
       </c>
       <c r="J15" s="2" t="s">
@@ -1579,12 +1597,12 @@
       <c r="M15" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="N15" s="26">
+      <c r="N15" s="24">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="27">
+      <c r="B16" s="25">
         <v>30</v>
       </c>
       <c r="C16" s="3" t="s">
@@ -1597,10 +1615,10 @@
       <c r="F16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G16" s="30">
+      <c r="G16" s="28">
         <v>29</v>
       </c>
-      <c r="I16" s="27">
+      <c r="I16" s="25">
         <v>30</v>
       </c>
       <c r="J16" s="2" t="s">
@@ -1611,12 +1629,12 @@
       <c r="M16" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="N16" s="26">
+      <c r="N16" s="24">
         <v>29</v>
       </c>
     </row>
     <row r="17" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="27">
+      <c r="B17" s="25">
         <v>32</v>
       </c>
       <c r="C17" s="3" t="s">
@@ -1629,10 +1647,10 @@
       <c r="F17" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G17" s="26">
+      <c r="G17" s="24">
         <v>31</v>
       </c>
-      <c r="I17" s="27">
+      <c r="I17" s="25">
         <v>32</v>
       </c>
       <c r="J17" s="2" t="s">
@@ -1643,12 +1661,12 @@
       <c r="M17" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="N17" s="26">
+      <c r="N17" s="24">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="27">
+      <c r="B18" s="25">
         <v>34</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1659,10 +1677,10 @@
       <c r="F18" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G18" s="26">
+      <c r="G18" s="24">
         <v>33</v>
       </c>
-      <c r="I18" s="27">
+      <c r="I18" s="25">
         <v>34</v>
       </c>
       <c r="J18" s="2" t="s">
@@ -1677,12 +1695,12 @@
       <c r="M18" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="N18" s="30">
+      <c r="N18" s="28">
         <v>33</v>
       </c>
     </row>
     <row r="19" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="29">
+      <c r="B19" s="27">
         <v>36</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -1697,10 +1715,10 @@
       <c r="F19" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G19" s="26">
+      <c r="G19" s="24">
         <v>35</v>
       </c>
-      <c r="I19" s="27">
+      <c r="I19" s="25">
         <v>36</v>
       </c>
       <c r="J19" s="2" t="s">
@@ -1711,12 +1729,12 @@
       <c r="M19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N19" s="26">
+      <c r="N19" s="24">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="2:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="29">
+      <c r="B20" s="27">
         <v>38</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -1731,10 +1749,10 @@
       <c r="F20" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G20" s="26">
+      <c r="G20" s="24">
         <v>37</v>
       </c>
-      <c r="I20" s="27">
+      <c r="I20" s="25">
         <v>38</v>
       </c>
       <c r="J20" s="2" t="s">
@@ -1745,7 +1763,7 @@
       <c r="M20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N20" s="26">
+      <c r="N20" s="24">
         <v>37</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sube los pines para esta versión, hay que terminar de configurarlos
</commit_message>
<xml_diff>
--- a/hardware/Circuito Final/Circuito externo/Pines controlador.xlsx
+++ b/hardware/Circuito Final/Circuito externo/Pines controlador.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="112">
   <si>
     <t>PC10</t>
   </si>
@@ -312,9 +312,6 @@
     <t>PD1</t>
   </si>
   <si>
-    <t>ADC4</t>
-  </si>
-  <si>
     <t>PA4</t>
   </si>
   <si>
@@ -515,6 +512,15 @@
   </si>
   <si>
     <t>S2</t>
+  </si>
+  <si>
+    <t>DEPURACIÓN</t>
+  </si>
+  <si>
+    <t>PROGRAMACIÓN</t>
+  </si>
+  <si>
+    <t>BOTON AZUL</t>
   </si>
 </sst>
 </file>
@@ -752,7 +758,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -806,17 +812,11 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1065,97 +1065,97 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="25">
+      <c r="B2" s="24">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" s="28" t="s">
         <v>105</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>106</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="24">
+      <c r="G2" s="23">
         <v>1</v>
       </c>
-      <c r="I2" s="25">
+      <c r="I2" s="24">
         <v>2</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="29" t="s">
+      <c r="K2" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="L2" s="28" t="s">
         <v>107</v>
-      </c>
-      <c r="L2" s="30" t="s">
-        <v>108</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="24">
+      <c r="N2" s="23">
         <v>1</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S2" s="21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="T2" s="21" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="25">
+      <c r="B3" s="24">
         <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="E3" s="14"/>
       <c r="F3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="24">
+      <c r="G3" s="23">
         <v>3</v>
       </c>
-      <c r="I3" s="25">
+      <c r="I3" s="24">
         <v>4</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="K3" s="12"/>
-      <c r="L3" s="31" t="s">
-        <v>109</v>
+      <c r="L3" s="29" t="s">
+        <v>108</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="N3" s="24">
+      <c r="N3" s="23">
         <v>3</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S3" s="21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="T3" s="21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="25">
+      <c r="B4" s="24">
         <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1166,10 +1166,10 @@
       <c r="F4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="24">
+      <c r="G4" s="23">
         <v>5</v>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="24">
         <v>6</v>
       </c>
       <c r="J4" s="2" t="s">
@@ -1177,26 +1177,26 @@
       </c>
       <c r="K4" s="12"/>
       <c r="L4" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N4" s="28">
+      <c r="N4" s="26">
         <v>5</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="S4" s="21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="T4" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="25">
+      <c r="B5" s="24">
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1207,10 +1207,10 @@
       <c r="F5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="23">
         <v>7</v>
       </c>
-      <c r="I5" s="25">
+      <c r="I5" s="24">
         <v>8</v>
       </c>
       <c r="J5" s="2" t="s">
@@ -1221,21 +1221,21 @@
       <c r="M5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N5" s="24">
+      <c r="N5" s="23">
         <v>7</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S5" s="21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="T5" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="25">
+      <c r="B6" s="24">
         <v>10</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -1246,10 +1246,10 @@
       <c r="F6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="23">
         <v>9</v>
       </c>
-      <c r="I6" s="25">
+      <c r="I6" s="24">
         <v>10</v>
       </c>
       <c r="J6" s="2" t="s">
@@ -1260,21 +1260,21 @@
       <c r="M6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="24">
+      <c r="N6" s="23">
         <v>9</v>
       </c>
       <c r="P6" s="8" t="s">
         <v>22</v>
       </c>
       <c r="S6" s="21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="T6" s="21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="25">
+      <c r="B7" s="24">
         <v>12</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -1285,135 +1285,137 @@
       <c r="F7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="23">
         <v>11</v>
       </c>
-      <c r="I7" s="27">
+      <c r="I7" s="25">
         <v>12</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="L7" s="23" t="s">
-        <v>79</v>
+        <v>100</v>
+      </c>
+      <c r="L7" s="29" t="s">
+        <v>5</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="N7" s="24">
+      <c r="N7" s="23">
         <v>11</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S7" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="T7" s="21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="25">
+      <c r="B8" s="24">
         <v>14</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="26"/>
+      <c r="D8" s="16" t="s">
+        <v>109</v>
+      </c>
       <c r="E8" s="14"/>
       <c r="F8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="23">
         <v>13</v>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="24">
         <v>14</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="K8" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="L8" s="23" t="s">
-        <v>78</v>
+      <c r="K8" s="15"/>
+      <c r="L8" s="29" t="s">
+        <v>37</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N8" s="24">
+      <c r="N8" s="23">
         <v>13</v>
       </c>
       <c r="S8" s="21" t="s">
         <v>5</v>
       </c>
       <c r="T8" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="25">
+      <c r="B9" s="24">
         <v>16</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="16"/>
+      <c r="D9" s="16" t="s">
+        <v>110</v>
+      </c>
       <c r="E9" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="23">
         <v>15</v>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="25">
         <v>16</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>26</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L9" s="14"/>
       <c r="M9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N9" s="24">
+      <c r="N9" s="23">
         <v>15</v>
       </c>
       <c r="S9" s="21" t="s">
         <v>37</v>
       </c>
       <c r="T9" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="25">
+      <c r="B10" s="24">
         <v>18</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="23">
         <v>17</v>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="24">
         <v>18</v>
       </c>
       <c r="J10" s="2" t="s">
@@ -1424,18 +1426,18 @@
       <c r="M10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N10" s="24">
+      <c r="N10" s="23">
         <v>17</v>
       </c>
       <c r="S10" s="21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="T10" s="21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="25">
+      <c r="B11" s="24">
         <v>20</v>
       </c>
       <c r="C11" s="11" t="s">
@@ -1446,10 +1448,10 @@
       <c r="F11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="23">
         <v>19</v>
       </c>
-      <c r="I11" s="25">
+      <c r="I11" s="24">
         <v>20</v>
       </c>
       <c r="J11" s="2" t="s">
@@ -1460,18 +1462,18 @@
       <c r="M11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="24">
+      <c r="N11" s="23">
         <v>19</v>
       </c>
       <c r="S11" s="21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="T11" s="21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="25">
+      <c r="B12" s="24">
         <v>22</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -1482,10 +1484,10 @@
       <c r="F12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="23">
         <v>21</v>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="24">
         <v>22</v>
       </c>
       <c r="J12" s="2" t="s">
@@ -1496,29 +1498,31 @@
       <c r="M12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="N12" s="24">
+      <c r="N12" s="23">
         <v>21</v>
       </c>
       <c r="T12" s="21" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="25">
+      <c r="B13" s="24">
         <v>24</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="26"/>
+      <c r="D13" s="16" t="s">
+        <v>111</v>
+      </c>
       <c r="E13" s="14"/>
       <c r="F13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="23">
         <v>23</v>
       </c>
-      <c r="I13" s="25">
+      <c r="I13" s="24">
         <v>24</v>
       </c>
       <c r="J13" s="2" t="s">
@@ -1529,15 +1533,15 @@
       <c r="M13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="N13" s="24">
+      <c r="N13" s="23">
         <v>23</v>
       </c>
       <c r="T13" s="21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="25">
+      <c r="B14" s="24">
         <v>26</v>
       </c>
       <c r="C14" s="11" t="s">
@@ -1548,10 +1552,10 @@
       <c r="F14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="23">
         <v>25</v>
       </c>
-      <c r="I14" s="25">
+      <c r="I14" s="24">
         <v>26</v>
       </c>
       <c r="J14" s="2" t="s">
@@ -1562,15 +1566,15 @@
       <c r="M14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="N14" s="24">
+      <c r="N14" s="23">
         <v>25</v>
       </c>
       <c r="T14" s="21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="25">
+      <c r="B15" s="24">
         <v>28</v>
       </c>
       <c r="C15" s="11" t="s">
@@ -1578,15 +1582,15 @@
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G15" s="28">
+      <c r="G15" s="26">
         <v>27</v>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="24">
         <v>28</v>
       </c>
       <c r="J15" s="2" t="s">
@@ -1597,12 +1601,12 @@
       <c r="M15" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="N15" s="24">
+      <c r="N15" s="23">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="25">
+      <c r="B16" s="24">
         <v>30</v>
       </c>
       <c r="C16" s="3" t="s">
@@ -1610,15 +1614,15 @@
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G16" s="28">
+      <c r="G16" s="26">
         <v>29</v>
       </c>
-      <c r="I16" s="25">
+      <c r="I16" s="24">
         <v>30</v>
       </c>
       <c r="J16" s="2" t="s">
@@ -1629,12 +1633,12 @@
       <c r="M16" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="N16" s="24">
+      <c r="N16" s="23">
         <v>29</v>
       </c>
     </row>
     <row r="17" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="25">
+      <c r="B17" s="24">
         <v>32</v>
       </c>
       <c r="C17" s="3" t="s">
@@ -1642,31 +1646,31 @@
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="23">
+        <v>31</v>
+      </c>
+      <c r="I17" s="24">
+        <v>32</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="G17" s="24">
-        <v>31</v>
-      </c>
-      <c r="I17" s="25">
-        <v>32</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="K17" s="12"/>
       <c r="L17" s="14"/>
       <c r="M17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="N17" s="24">
+        <v>55</v>
+      </c>
+      <c r="N17" s="23">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="25">
+      <c r="B18" s="24">
         <v>34</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1675,95 +1679,95 @@
       <c r="D18" s="12"/>
       <c r="E18" s="22"/>
       <c r="F18" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G18" s="23">
+        <v>33</v>
+      </c>
+      <c r="I18" s="24">
+        <v>34</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G18" s="24">
+      <c r="K18" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="L18" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="N18" s="26">
         <v>33</v>
       </c>
-      <c r="I18" s="25">
-        <v>34</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="K18" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="L18" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="M18" s="2" t="s">
+    </row>
+    <row r="19" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="25">
+        <v>36</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="N18" s="28">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="27">
+      <c r="D19" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" s="23">
+        <v>35</v>
+      </c>
+      <c r="I19" s="24">
         <v>36</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="F19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="G19" s="24">
-        <v>35</v>
-      </c>
-      <c r="I19" s="25">
-        <v>36</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="K19" s="12"/>
       <c r="L19" s="14"/>
       <c r="M19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N19" s="24">
+      <c r="N19" s="23">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="2:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="27">
+      <c r="B20" s="25">
         <v>38</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="19" t="s">
-        <v>98</v>
-      </c>
-      <c r="E20" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="F20" s="2" t="s">
+      <c r="G20" s="23">
+        <v>37</v>
+      </c>
+      <c r="I20" s="24">
+        <v>38</v>
+      </c>
+      <c r="J20" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="G20" s="24">
-        <v>37</v>
-      </c>
-      <c r="I20" s="25">
-        <v>38</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="K20" s="17"/>
       <c r="L20" s="18"/>
       <c r="M20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N20" s="24">
+      <c r="N20" s="23">
         <v>37</v>
       </c>
     </row>

</xml_diff>

<commit_message>
acomoda los pines en el excel de pines
</commit_message>
<xml_diff>
--- a/hardware/Circuito Final/Circuito externo/Pines controlador.xlsx
+++ b/hardware/Circuito Final/Circuito externo/Pines controlador.xlsx
@@ -1364,9 +1364,7 @@
         <v>25</v>
       </c>
       <c r="D9" s="16"/>
-      <c r="E9" s="14" t="s">
-        <v>93</v>
-      </c>
+      <c r="E9" s="14"/>
       <c r="F9" s="2" t="s">
         <v>18</v>
       </c>
@@ -1403,10 +1401,10 @@
       <c r="C10" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" s="14"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="14" t="s">
+        <v>93</v>
+      </c>
       <c r="F10" s="2" t="s">
         <v>29</v>
       </c>
@@ -1510,7 +1508,9 @@
       <c r="C13" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="26"/>
+      <c r="D13" s="26" t="s">
+        <v>37</v>
+      </c>
       <c r="E13" s="14"/>
       <c r="F13" s="2" t="s">
         <v>38</v>

</xml_diff>